<commit_message>
PCB updated - cosmetics
</commit_message>
<xml_diff>
--- a/system_design/Georgetown/V0.5/bill_of_materials/bill_of_materials.xlsx
+++ b/system_design/Georgetown/V0.5/bill_of_materials/bill_of_materials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emailsc-my.sharepoint.com/personal/asifuzzaman_sc_edu/Documents/Github Repos/UAV-Deployable-Stage-Height-Sensor/system_design/Georgetown/V0.5/bill_of_materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="13_ncr:1_{68C7DE68-14CC-422B-B4F0-50A88173269E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7043877E-A105-466F-B8FC-6AD2D7514B58}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="13_ncr:1_{68C7DE68-14CC-422B-B4F0-50A88173269E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{152FAEFB-A4BB-469B-BA28-EC4D5D003E9E}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -233,9 +233,6 @@
     <t>https://www.digikey.com/en/products/detail/c-k/JS202011CQN/1640097</t>
   </si>
   <si>
-    <t>RES SMD (100, 1k, 2K, 4.7k) OHM 1% 1/4W 1206</t>
-  </si>
-  <si>
     <t xml:space="preserve"> C1206S104K5RACAUTO 0.1 uF 10% 50V Ceramic Capacitor X7R 1206 (3216 Metric)</t>
   </si>
   <si>
@@ -294,6 +291,9 @@
   </si>
   <si>
     <t>B3B-XH-A</t>
+  </si>
+  <si>
+    <t>RES SMD (1k, 2K, 4.7k) OHM 1% 1/4W 1206</t>
   </si>
 </sst>
 </file>
@@ -733,10 +733,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -748,7 +748,7 @@
         <v>2.5</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -1016,7 +1016,7 @@
         <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="C17">
         <v>7</v>
@@ -1053,10 +1053,10 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B19" t="s">
         <v>68</v>
-      </c>
-      <c r="B19" t="s">
-        <v>69</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1068,15 +1068,15 @@
         <v>0.4</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1088,15 +1088,15 @@
         <v>0.2</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C21">
         <v>4</v>
@@ -1119,13 +1119,13 @@
         <v>28</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22">
         <v>3.58</v>
       </c>
       <c r="E22">
-        <v>7.16</v>
+        <v>3.58</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>58</v>
@@ -1193,10 +1193,10 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -1208,15 +1208,15 @@
         <v>2.15</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B27" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -1228,15 +1228,15 @@
         <v>0.13</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C28">
         <v>9</v>
@@ -1248,7 +1248,7 @@
         <v>66.510000000000005</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="B30">
         <f>SUM(E2:E28)</f>
-        <v>180.49500000000003</v>
+        <v>176.91500000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Diode added in BOM and CAD folder cleaned
</commit_message>
<xml_diff>
--- a/system_design/Georgetown/V0.5/bill_of_materials/bill_of_materials.xlsx
+++ b/system_design/Georgetown/V0.5/bill_of_materials/bill_of_materials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emailsc-my.sharepoint.com/personal/asifuzzaman_sc_edu/Documents/Github Repos/UAV-Deployable-Stage-Height-Sensor/system_design/Georgetown/V0.5/bill_of_materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="13_ncr:1_{68C7DE68-14CC-422B-B4F0-50A88173269E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{152FAEFB-A4BB-469B-BA28-EC4D5D003E9E}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{68C7DE68-14CC-422B-B4F0-50A88173269E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7C7C9A8-1D10-4453-9B45-A2BEE11E1D62}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="89">
   <si>
     <t>Arduino Nano</t>
   </si>
@@ -294,6 +294,15 @@
   </si>
   <si>
     <t>RES SMD (1k, 2K, 4.7k) OHM 1% 1/4W 1206</t>
+  </si>
+  <si>
+    <t>Schottky Diode</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/onsemi/BAT54T1G/918319</t>
+  </si>
+  <si>
+    <t>BAT54T1G</t>
   </si>
 </sst>
 </file>
@@ -680,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
@@ -1053,214 +1062,234 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
       <c r="D19">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="E19">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E20">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C21">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D21">
-        <v>0.42</v>
+        <v>1</v>
       </c>
       <c r="E21">
-        <v>1.68</v>
+        <v>0.2</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D22">
-        <v>3.58</v>
+        <v>0.42</v>
       </c>
       <c r="E22">
-        <v>3.58</v>
+        <v>1.68</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23">
-        <v>6.54</v>
+        <v>3.58</v>
       </c>
       <c r="E23">
-        <v>6.54</v>
+        <v>3.58</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
       <c r="D24">
-        <v>1.05</v>
+        <v>6.54</v>
       </c>
       <c r="E24">
-        <v>1.05</v>
+        <v>6.54</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
       <c r="D25">
-        <v>0.91</v>
+        <v>1.05</v>
       </c>
       <c r="E25">
-        <v>0.91</v>
+        <v>1.05</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26">
-        <v>2.15</v>
+        <v>0.91</v>
       </c>
       <c r="E26">
-        <v>2.15</v>
+        <v>0.91</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B27" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
       <c r="D27">
-        <v>0.13</v>
+        <v>2.15</v>
       </c>
       <c r="E27">
-        <v>0.13</v>
+        <v>2.15</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>0.13</v>
+      </c>
+      <c r="E28">
+        <v>0.13</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>79</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>81</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>9</v>
       </c>
-      <c r="D28">
+      <c r="D29">
         <v>7.39</v>
       </c>
-      <c r="E28">
+      <c r="E29">
         <v>66.510000000000005</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="F29" s="1"/>
-    </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>36</v>
       </c>
-      <c r="B30">
-        <f>SUM(E2:E28)</f>
-        <v>176.91500000000002</v>
+      <c r="B31">
+        <f>SUM(E2:E29)</f>
+        <v>177.01500000000004</v>
       </c>
     </row>
   </sheetData>
@@ -1279,20 +1308,21 @@
     <hyperlink ref="F16" r:id="rId12" display="https://www.digikey.com/en/products/detail/american-opto-plus-led/L314ED/13677700?s=N4IgTCBcDaIDIGYCMAWAogERAXQL5A" xr:uid="{EB1FB783-CD78-4F2E-ADAE-2EFC2E0C050D}"/>
     <hyperlink ref="F17" r:id="rId13" xr:uid="{1CE23A94-3355-4CE3-BD99-944097BF2C76}"/>
     <hyperlink ref="F18" r:id="rId14" display="https://www.digikey.com/en/products/detail/panasonic-electronic-components/ERJ-8BSJR10V/5647718?s=N4IgTCBcDaIKICUBSBaAHAIQMpIQRgAYA1AAgTixIIDo8SB5ACQFkSBWAHQ4FIS8B6MAHU%2BYAgDYQAXQC%2BQA" xr:uid="{435BBBC4-E5AA-4343-9940-0DAF3E021F72}"/>
-    <hyperlink ref="F21" r:id="rId15" display="https://www.digikey.com/en/products/detail/kemet/c1206s104k5racauto/10232834" xr:uid="{CDDFAE49-11BE-4283-9E44-D17951ACE335}"/>
-    <hyperlink ref="F22" r:id="rId16" display="https://www.digikey.com/en/products/detail/microchip-technology/mic5239-5-0ys-tr/2346595" xr:uid="{0FF0C8FA-B521-42B4-9637-4551CDF56AE0}"/>
-    <hyperlink ref="F23" r:id="rId17" display="https://www.grainger.com/product/Pipe-PVC-1ABA1" xr:uid="{98BE1843-601E-422A-8251-9162A4C6D813}"/>
-    <hyperlink ref="F24" r:id="rId18" display="https://www.digikey.com/en/products/detail/sparkfun-electronics/PRT-11864/6818769?s=N4IgTCBcDaIAoCUAqBaAjGgHANgCwgF0BfIA" xr:uid="{2FC61876-0275-459F-BE77-C7067ECA8C84}"/>
-    <hyperlink ref="F25" r:id="rId19" display="https://www.digikey.com/en/products/detail/samtec-inc/ssa-104-w-t/1105908" xr:uid="{5CEFEAD0-E765-4C5C-8B17-4D481AAEE74F}"/>
+    <hyperlink ref="F22" r:id="rId15" display="https://www.digikey.com/en/products/detail/kemet/c1206s104k5racauto/10232834" xr:uid="{CDDFAE49-11BE-4283-9E44-D17951ACE335}"/>
+    <hyperlink ref="F23" r:id="rId16" display="https://www.digikey.com/en/products/detail/microchip-technology/mic5239-5-0ys-tr/2346595" xr:uid="{0FF0C8FA-B521-42B4-9637-4551CDF56AE0}"/>
+    <hyperlink ref="F24" r:id="rId17" display="https://www.grainger.com/product/Pipe-PVC-1ABA1" xr:uid="{98BE1843-601E-422A-8251-9162A4C6D813}"/>
+    <hyperlink ref="F25" r:id="rId18" display="https://www.digikey.com/en/products/detail/sparkfun-electronics/PRT-11864/6818769?s=N4IgTCBcDaIAoCUAqBaAjGgHANgCwgF0BfIA" xr:uid="{2FC61876-0275-459F-BE77-C7067ECA8C84}"/>
+    <hyperlink ref="F26" r:id="rId19" display="https://www.digikey.com/en/products/detail/samtec-inc/ssa-104-w-t/1105908" xr:uid="{5CEFEAD0-E765-4C5C-8B17-4D481AAEE74F}"/>
     <hyperlink ref="F13" r:id="rId20" xr:uid="{98CBDFFF-5BC0-4691-985C-193C55CD2A4F}"/>
     <hyperlink ref="F15" r:id="rId21" xr:uid="{F40F3420-CF30-4700-92F3-040B50F37E84}"/>
-    <hyperlink ref="F19" r:id="rId22" xr:uid="{CF84383E-32DC-4F7A-8B1F-D5487EDC174E}"/>
-    <hyperlink ref="F20" r:id="rId23" xr:uid="{9AFC6348-0E57-4A67-A197-41D4FD45794D}"/>
+    <hyperlink ref="F20" r:id="rId22" xr:uid="{CF84383E-32DC-4F7A-8B1F-D5487EDC174E}"/>
+    <hyperlink ref="F21" r:id="rId23" xr:uid="{9AFC6348-0E57-4A67-A197-41D4FD45794D}"/>
     <hyperlink ref="F3" r:id="rId24" xr:uid="{132AA37F-9E12-44EF-9546-36BDCE2F9F6B}"/>
-    <hyperlink ref="F28" r:id="rId25" xr:uid="{BECD5DE6-8852-4EA8-869E-7E18A46D5C74}"/>
-    <hyperlink ref="F27" r:id="rId26" display="https://www.digikey.com/en/products/detail/jst-sales-america-inc/B3B-XH-A/1651046?gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLlgCz6Py2S0va5_igHe8YH5kP&amp;gclid=Cj0KCQjwuvrBBhDcARIsAKRrkjelT39dppIYbNMYGQDQKVRAcVAnRo2gDZvSJK6NkGomAkksSe1uUHcaAmLSEALw_wcB&amp;gclsrc=aw.ds" xr:uid="{9BDFB2BD-EFF6-4DEE-BBC3-2D01594D0DB0}"/>
+    <hyperlink ref="F29" r:id="rId25" xr:uid="{BECD5DE6-8852-4EA8-869E-7E18A46D5C74}"/>
+    <hyperlink ref="F28" r:id="rId26" display="https://www.digikey.com/en/products/detail/jst-sales-america-inc/B3B-XH-A/1651046?gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLlgCz6Py2S0va5_igHe8YH5kP&amp;gclid=Cj0KCQjwuvrBBhDcARIsAKRrkjelT39dppIYbNMYGQDQKVRAcVAnRo2gDZvSJK6NkGomAkksSe1uUHcaAmLSEALw_wcB&amp;gclsrc=aw.ds" xr:uid="{9BDFB2BD-EFF6-4DEE-BBC3-2D01594D0DB0}"/>
+    <hyperlink ref="F19" r:id="rId27" xr:uid="{4FB5C311-0780-4C35-9E62-7B63EE0B1C7F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId27"/>
+  <pageSetup orientation="portrait" r:id="rId28"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
PCB tray design updated
</commit_message>
<xml_diff>
--- a/system_design/Georgetown/V0.5/bill_of_materials/bill_of_materials.xlsx
+++ b/system_design/Georgetown/V0.5/bill_of_materials/bill_of_materials.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{79DF5EF5-95A3-3841-BD8C-059FB5CD78EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DF03F03-B2E1-4173-A4FA-07851DC7CB47}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-120" yWindow="-16455" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>

</xml_diff>